<commit_message>
Record discovered encodings in v2 dictionary (suicide-method items + notes)
Sync the ground-truth dictionary with the rules implemented in rules.py:

- 7 SUICIDE method/lethality items (ltsv02/04/05/06, ltsg03/05/06): replace the
  stale copy-pasted cells (which wrongly said "recode to {1=Oui,0=Non}" or
  carried the deleted timing-items' findings) with the actual Beck/Columbia
  medical-lethality ordinal mapping, set the correct Final dtype, and add sanity
  bounds matching the code ranges (e.g. ltsg05 [0,6]; 6=Mort). QA confirms the
  bounds reject no real data (211/211 pass).
- qt/rr/qtc/edulevel/siteid_city: append an implementation pointer to the Rule
  cell (rules.py:: function, v2-gated) so the dictionary records where each
  harmonization lives.

Verified: dictionary loads (216 vars); 92 tests pass; qa_harmonization 211/211.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/face-common-vars-v2.xlsx
+++ b/data/face-common-vars-v2.xlsx
@@ -1587,7 +1587,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Derive canonical site from fondacode leading digits; map to city via data/site_lookup.csv. Use as ComBat batch / site confound.</t>
+          <t>Derive canonical site from fondacode leading digits; map to city via data/site_lookup.csv. Use as ComBat batch / site confound. | Implemented in rules.py::derive_siteid_city (fondacode leading digits + data/site_lookup.csv).</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>Verify units: mmHg for BP, msec for QT/QTc, bpm for HR, kg for weight, cm for height. Convert if any source uses different.</t>
+          <t>Verify units: mmHg for BP, msec for QT/QTc, bpm for HR, kg for weight, cm for height. Convert if any source uses different. | Implemented in rules.py::qt (ms→s: value&gt;5 ⇒ /1000), v2-gated. Bound in seconds.</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Verify units: mmHg for BP, msec for QT/QTc, bpm for HR, kg for weight, cm for height. Convert if any source uses different.</t>
+          <t>Verify units: mmHg for BP, msec for QT/QTc, bpm for HR, kg for weight, cm for height. Convert if any source uses different. | Implemented in rules.py::rr (ms→s: value&gt;5 ⇒ /1000), v2-gated. Bound in seconds.</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -5679,6 +5679,11 @@
       <c r="N67" s="22" t="inlineStr">
         <is>
           <t>3 (BP/SZ/DR)</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>Implemented in rules.py::qtc (ms→s: value&gt;5 ⇒ /1000), v2-gated. Bound in seconds.</t>
         </is>
       </c>
     </row>
@@ -10774,11 +10779,15 @@
       </c>
       <c r="F136" s="20" t="inlineStr">
         <is>
-          <t>NUM (mètres)</t>
-        </is>
-      </c>
-      <c r="G136" s="100" t="n"/>
-      <c r="H136" s="129" t="n"/>
+          <t>Ordinal jump height: 1=Hauteur d'homme, 2=Hauteur modérée, 3=D'un endroit élevé.</t>
+        </is>
+      </c>
+      <c r="G136" s="100" t="n">
+        <v>1</v>
+      </c>
+      <c r="H136" s="129" t="n">
+        <v>3</v>
+      </c>
       <c r="I136" s="20" t="inlineStr">
         <is>
           <t>Jump height : objective lethality marker when the method is jumping; correlates with lethal intent and injury severity.</t>
@@ -10811,12 +10820,12 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>Recode all to {1=Oui, 0=Non, NA=missing}. BP/SZ: 'Oui'→1, 'Non'→0. DR: already numeric, no change needed.</t>
+          <t>rules.py::ltsv02 — BP text → ordinal 1-3; DR codes pass through; SZ absent.</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>✓ CONFIRMED in data: BP and SZ store as text {'Oui','Non'}; DR stores as numeric {0,1}. ~30%-72% missing depending on pathology.</t>
+          <t>Jump height (LTSV02). BP stores French text, DR is pre-numericized, SZ does not collect it. Encoded in rules.py (v2-gated; v1 unchanged). Verified by scripts/qa_harmonization.py.</t>
         </is>
       </c>
     </row>
@@ -10914,11 +10923,15 @@
       </c>
       <c r="F138" s="20" t="inlineStr">
         <is>
-          <t>Categorical (Columbia lethality)</t>
-        </is>
-      </c>
-      <c r="G138" s="100" t="n"/>
-      <c r="H138" s="129" t="n"/>
+          <t>Firearm lethality (Columbia): 0=Pas de dommage, 2=extrémité, 5=abdomen/thorax.</t>
+        </is>
+      </c>
+      <c r="G138" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H138" s="129" t="n">
+        <v>6</v>
+      </c>
       <c r="I138" s="20" t="inlineStr">
         <is>
           <t>Lethality grading for firearm : the highest case-fatality method; lethality grade refines the severity of the violent-method phenotype.</t>
@@ -10951,12 +10964,12 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>Reclassify as PARTIAL. Pool BP+DR; SZ NA.</t>
+          <t>rules.py::ltsv04 — BP text → Beck/Columbia medical-lethality ordinal (0=no damage → higher=more severe → death). DR codes pass through; SZ absent.</t>
         </is>
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>LTSV04 (Létalité si méthode = Arme à feu). Same situation as R150.</t>
+          <t>Firearm lethality (LTSV04). BP stores French text, DR is pre-numericized, SZ does not collect it. Encoded in rules.py (v2-gated; v1 unchanged). Verified by scripts/qa_harmonization.py.</t>
         </is>
       </c>
     </row>
@@ -10984,11 +10997,15 @@
       </c>
       <c r="F139" s="20" t="inlineStr">
         <is>
-          <t>Categorical (Columbia lethality)</t>
-        </is>
-      </c>
-      <c r="G139" s="100" t="n"/>
-      <c r="H139" s="129" t="n"/>
+          <t>Self-immolation lethality (Columbia): 0=no damage, 1=1st°, 2=2nd°, 4=3rd° burns.</t>
+        </is>
+      </c>
+      <c r="G139" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H139" s="129" t="n">
+        <v>6</v>
+      </c>
       <c r="I139" s="20" t="inlineStr">
         <is>
           <t>Lethality grading for immolation : rare but high-lethality method, often associated with severe psychotic features or extreme distress.</t>
@@ -10996,7 +11013,7 @@
       </c>
       <c r="J139" s="20" t="inlineStr">
         <is>
-          <t>int8 categorical</t>
+          <t>int8 ordinal</t>
         </is>
       </c>
       <c r="K139" s="20" t="inlineStr">
@@ -11021,12 +11038,12 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>Map BP/SZ text → numeric: {'La semaine dernière'→0, 'Il y a entre une semaine et la dernière visite'→0 (collapse to la semaine dernière, OR keep as 0.5 if you want to preserve granularity for BP/SZ-only sub-analyses), 'Il y a entre deux semaines et douze mois'→1, 'Il y a plus d''un an'→2}. DR is already 0/1/2 — no change. Document the BP/SZ 4-to-3 collapse choice.</t>
+          <t>rules.py::ltsv05 — BP text → Beck/Columbia medical-lethality ordinal (0=no damage → higher=more severe → death). DR codes pass through; SZ absent.</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>⚠ REVISED finding: data shows BP and SZ have 4 timing categories — 'La semaine dernière', 'Il y a entre une semaine et la dernière visite' (extra visit-context category), 'Il y a entre deux semaines et douze mois', 'Il y a plus d''un an'. DR has only 3 categories (0/1/2 = la semaine dernière / 2 sem-12 mois / &gt;1 an), MISSING the 'Il y a entre une semaine et la dernière visite' category. The thesaurus's off-by-one suspicion was wrong; the real issue is category granularity.</t>
+          <t>Immolation lethality (LTSV05). BP stores French text, DR is pre-numericized, SZ does not collect it. Encoded in rules.py (v2-gated; v1 unchanged). Verified by scripts/qa_harmonization.py.</t>
         </is>
       </c>
     </row>
@@ -11054,11 +11071,15 @@
       </c>
       <c r="F140" s="20" t="inlineStr">
         <is>
-          <t>Categorical (Columbia lethality)</t>
-        </is>
-      </c>
-      <c r="G140" s="100" t="n"/>
-      <c r="H140" s="129" t="n"/>
+          <t>Drowning lethality (Columbia): 0=no damage, 2=conscious/mild, 4=unconscious.</t>
+        </is>
+      </c>
+      <c r="G140" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" s="129" t="n">
+        <v>6</v>
+      </c>
       <c r="I140" s="20" t="inlineStr">
         <is>
           <t>Lethality grading for drowning : method-specific severity refinement complementing the categorical method variable.</t>
@@ -11091,12 +11112,12 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>Recode all to {1=Oui, 0=Non, NA=missing}. BP/SZ: 'Oui'→1, 'Non'→0. DR: already numeric, no change needed.</t>
+          <t>rules.py::ltsv06 — BP text → Beck/Columbia medical-lethality ordinal (0=no damage → higher=more severe → death). DR codes pass through; SZ absent.</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>✓ CONFIRMED in data: BP and SZ store as text {'Oui','Non'}; DR stores as numeric {0,1}. ~30%-72% missing depending on pathology.</t>
+          <t>Drowning lethality (LTSV06). BP stores French text, DR is pre-numericized, SZ does not collect it. Encoded in rules.py (v2-gated; v1 unchanged). Verified by scripts/qa_harmonization.py.</t>
         </is>
       </c>
     </row>
@@ -11404,11 +11425,15 @@
       </c>
       <c r="F145" s="20" t="inlineStr">
         <is>
-          <t>Categorical</t>
-        </is>
-      </c>
-      <c r="G145" s="100" t="n"/>
-      <c r="H145" s="129" t="n"/>
+          <t>Non-sedative drug type: 1=OTC, 2=non-psychotrope Rx, 3=other ingested, 5=lithium; Inconnu→NA.</t>
+        </is>
+      </c>
+      <c r="G145" s="100" t="n">
+        <v>1</v>
+      </c>
+      <c r="H145" s="129" t="n">
+        <v>8</v>
+      </c>
       <c r="I145" s="20" t="inlineStr">
         <is>
           <t>Non-sedative drug class used : complements the sedative-class variable for full pharmacologic characterisation of the overdose.</t>
@@ -11441,12 +11466,12 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>Map BP/SZ text → numeric: {'La semaine dernière'→0, 'Il y a entre une semaine et la dernière visite'→0 (collapse to la semaine dernière, OR keep as 0.5 if you want to preserve granularity for BP/SZ-only sub-analyses), 'Il y a entre deux semaines et douze mois'→1, 'Il y a plus d''un an'→2}. DR is already 0/1/2 — no change. Document the BP/SZ 4-to-3 collapse choice.</t>
+          <t>rules.py::ltsg03 — BP text → category code; DR codes pass through; SZ absent.</t>
         </is>
       </c>
       <c r="P145" t="inlineStr">
         <is>
-          <t>⚠ REVISED finding: data shows BP and SZ have 4 timing categories — 'La semaine dernière', 'Il y a entre une semaine et la dernière visite' (extra visit-context category), 'Il y a entre deux semaines et douze mois', 'Il y a plus d''un an'. DR has only 3 categories (0/1/2 = la semaine dernière / 2 sem-12 mois / &gt;1 an), MISSING the 'Il y a entre une semaine et la dernière visite' category. The thesaurus's off-by-one suspicion was wrong; the real issue is category granularity.</t>
+          <t>Non-sedative drug type in overdose (LTSG03). BP stores French text, DR is pre-numericized, SZ does not collect it. Encoded in rules.py (v2-gated; v1 unchanged). Verified by scripts/qa_harmonization.py.</t>
         </is>
       </c>
     </row>
@@ -11544,11 +11569,15 @@
       </c>
       <c r="F147" s="20" t="inlineStr">
         <is>
-          <t>Categorical (Columbia lethality)</t>
-        </is>
-      </c>
-      <c r="G147" s="100" t="n"/>
-      <c r="H147" s="129" t="n"/>
+          <t>Medication-overdose lethality (Columbia): 0=none/minimal … 4=major systemic, 6=Mort.</t>
+        </is>
+      </c>
+      <c r="G147" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" s="129" t="n">
+        <v>6</v>
+      </c>
       <c r="I147" s="20" t="inlineStr">
         <is>
           <t>Lethality grading for non-sedative medication overdose : complements LTSG04 for full toxicological lethality phenotype.</t>
@@ -11556,7 +11585,7 @@
       </c>
       <c r="J147" s="20" t="inlineStr">
         <is>
-          <t>int8 categorical</t>
+          <t>int8 ordinal</t>
         </is>
       </c>
       <c r="K147" s="20" t="inlineStr">
@@ -11581,12 +11610,12 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>Map BP/SZ text → numeric: {'La semaine dernière'→0, 'Il y a entre une semaine et la dernière visite'→0 (collapse to la semaine dernière, OR keep as 0.5 if you want to preserve granularity for BP/SZ-only sub-analyses), 'Il y a entre deux semaines et douze mois'→1, 'Il y a plus d''un an'→2}. DR is already 0/1/2 — no change. Document the BP/SZ 4-to-3 collapse choice.</t>
+          <t>rules.py::ltsg05 — BP text → Beck/Columbia medical-lethality ordinal (0=no damage → higher=more severe → death). DR codes pass through; SZ absent.</t>
         </is>
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>⚠ REVISED finding: data shows BP and SZ have 4 timing categories — 'La semaine dernière', 'Il y a entre une semaine et la dernière visite' (extra visit-context category), 'Il y a entre deux semaines et douze mois', 'Il y a plus d''un an'. DR has only 3 categories (0/1/2 = la semaine dernière / 2 sem-12 mois / &gt;1 an), MISSING the 'Il y a entre une semaine et la dernière visite' category. The thesaurus's off-by-one suspicion was wrong; the real issue is category granularity.</t>
+          <t>Overdose lethality (LTSG05). BP stores French text, DR is pre-numericized, SZ does not collect it. Encoded in rules.py (v2-gated; v1 unchanged). Verified by scripts/qa_harmonization.py.</t>
         </is>
       </c>
     </row>
@@ -11614,11 +11643,15 @@
       </c>
       <c r="F148" s="20" t="inlineStr">
         <is>
-          <t>Categorical (Columbia lethality)</t>
-        </is>
-      </c>
-      <c r="G148" s="100" t="n"/>
-      <c r="H148" s="129" t="n"/>
+          <t>Phlebotomy (cutting) lethality (Columbia): 1=scratches … 4=major blood loss/transfusion.</t>
+        </is>
+      </c>
+      <c r="G148" s="100" t="n">
+        <v>1</v>
+      </c>
+      <c r="H148" s="129" t="n">
+        <v>6</v>
+      </c>
       <c r="I148" s="20" t="inlineStr">
         <is>
           <t>Lethality grading for self-cutting : separates non-suicidal self-injury from genuine suicidal phlebotomy on medical severity grounds.</t>
@@ -11626,7 +11659,7 @@
       </c>
       <c r="J148" s="20" t="inlineStr">
         <is>
-          <t>int8 categorical</t>
+          <t>int8 ordinal</t>
         </is>
       </c>
       <c r="K148" s="20" t="inlineStr">
@@ -11651,12 +11684,12 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>Recode all to {1=Oui, 0=Non, NA=missing}. BP/SZ: 'Oui'→1, 'Non'→0. DR: already numeric, no change needed.</t>
+          <t>rules.py::ltsg06 — BP text → Beck/Columbia medical-lethality ordinal (0=no damage → higher=more severe → death). DR codes pass through; SZ absent.</t>
         </is>
       </c>
       <c r="P148" t="inlineStr">
         <is>
-          <t>✓ CONFIRMED in data: BP and SZ store as text {'Oui','Non'}; DR stores as numeric {0,1}. ~30%-72% missing depending on pathology.</t>
+          <t>Phlebotomy lethality (LTSG06). BP stores French text, DR is pre-numericized, SZ does not collect it. Encoded in rules.py (v2-gated; v1 unchanged). Verified by scripts/qa_harmonization.py.</t>
         </is>
       </c>
     </row>
@@ -16415,7 +16448,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>Recode both BP and SZ: 'BAC' → 12 (baccalauréat = end of lycée, after 12 years of schooling); other numeric strings → cast to int. Verify other rare strings ('BEP', 'CAP', etc.) per-cohort and apply the thesaurus mapping (CP-CM2=1-5, collège=6-9, lycée=10-12, CAP=13, BEP=14, BAC+1 to BAC+5=15-19, Doctorat=20). DR is ready to pool directly.</t>
+          <t>Recode both BP and SZ: 'BAC' → 12 (baccalauréat = end of lycée, after 12 years of schooling); other numeric strings → cast to int. Verify other rare strings ('BEP', 'CAP', etc.) per-cohort and apply the thesaurus mapping (CP-CM2=1-5, collège=6-9, lycée=10-12, CAP=13, BEP=14, BAC+1 to BAC+5=15-19, Doctorat=20). DR is ready to pool directly. | Implemented in rules.py::edulevel (SZ text tokens BAC/CAP/Doctorat→ordinal), v2-gated.</t>
         </is>
       </c>
       <c r="P214" t="inlineStr">

</xml_diff>